<commit_message>
Upload invest-law.eu : détection des doublons par le mois du nom du rapport, procédure mise à jour
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T5bmrEsYEKdmqU5ckZhZrJ
</commit_message>
<xml_diff>
--- a/INVESTLAW/MANIFEST_UPLOAD.xlsx
+++ b/INVESTLAW/MANIFEST_UPLOAD.xlsx
@@ -606,12 +606,12 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>A_UPLOADER</t>
+          <t>A_VERIFIER</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2 rapport(s) existant(s)</t>
+          <t>rapport de gestion (2026-09-28)</t>
         </is>
       </c>
     </row>
@@ -651,6 +651,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J4" t="n">
         <v>211</v>
       </c>
@@ -761,6 +766,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J6" t="n">
         <v>277</v>
       </c>
@@ -816,6 +826,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J7" t="n">
         <v>219</v>
       </c>
@@ -871,6 +886,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J8" t="n">
         <v>275</v>
       </c>
@@ -981,6 +1001,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J10" t="n">
         <v>529</v>
       </c>
@@ -991,12 +1016,12 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-30)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -1311,6 +1336,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J16" t="n">
         <v>410</v>
       </c>
@@ -1366,6 +1396,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J17" t="n">
         <v>42</v>
       </c>
@@ -1376,12 +1411,12 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>DIC (Document d'informations clés) (2026-09-30); Rapport de gestion Août 2026 (2026-09-30)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -1491,12 +1526,12 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>A_UPLOADER</t>
+          <t>PLUS_RECENT_PRESENT</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>2 rapport(s) existant(s)</t>
+          <t>Rapport de gestion Août 2026 (2026-09-30)</t>
         </is>
       </c>
     </row>
@@ -1536,6 +1571,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J20" t="n">
         <v>26</v>
       </c>
@@ -1546,12 +1586,12 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-30)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -1646,6 +1686,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J22" t="n">
         <v>515</v>
       </c>
@@ -1656,12 +1701,12 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-30)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -1701,6 +1746,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J23" t="n">
         <v>215</v>
       </c>
@@ -1711,12 +1761,12 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>DIC (Document d'informations clés) (2026-09-30); Rapport de gestion Mai 2024 (2026-09-30)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -1756,6 +1806,11 @@
           <t>ES</t>
         </is>
       </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J24" t="n">
         <v>3</v>
       </c>
@@ -1766,12 +1821,12 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>DIC (Document d'informations clés) (2026-09-30); Rapport de gestion Août 2026 (2026-09-30)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -1826,12 +1881,12 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>A_UPLOADER</t>
+          <t>PLUS_RECENT_PRESENT</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>2 rapport(s) existant(s)</t>
+          <t>Rapport de gestion Août 2026 (2026-09-30)</t>
         </is>
       </c>
     </row>
@@ -1871,6 +1926,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J26" t="n">
         <v>46</v>
       </c>
@@ -1926,6 +1986,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J27" t="n">
         <v>220</v>
       </c>
@@ -1981,6 +2046,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J28" t="n">
         <v>82</v>
       </c>
@@ -2036,6 +2106,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J29" t="n">
         <v>72</v>
       </c>
@@ -2091,6 +2166,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J30" t="n">
         <v>222</v>
       </c>
@@ -2146,6 +2226,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J31" t="n">
         <v>221</v>
       </c>
@@ -2531,6 +2616,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J38" t="n">
         <v>231</v>
       </c>
@@ -2541,12 +2631,12 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>DIC (Document d'informations clés) (2026-09-30); Rapport de gestion Janvier 2026 (2026-09-30)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -2586,6 +2676,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J39" t="n">
         <v>230</v>
       </c>
@@ -3521,6 +3616,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J56" t="n">
         <v>245</v>
       </c>
@@ -3576,6 +3676,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J57" t="n">
         <v>246</v>
       </c>
@@ -3631,6 +3736,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J58" t="n">
         <v>247</v>
       </c>
@@ -3686,6 +3796,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J59" t="n">
         <v>12</v>
       </c>
@@ -3741,6 +3856,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J60" t="n">
         <v>243</v>
       </c>
@@ -3796,6 +3916,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J61" t="n">
         <v>244</v>
       </c>
@@ -3856,6 +3981,11 @@
           <t>Fiche du fonds sans ISIN de la part (multi-parts)</t>
         </is>
       </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J62" t="n">
         <v>491</v>
       </c>
@@ -4021,6 +4151,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J65" t="n">
         <v>255</v>
       </c>
@@ -4241,6 +4376,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J69" t="n">
         <v>87</v>
       </c>
@@ -4251,12 +4391,12 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-10)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -4296,6 +4436,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J70" t="n">
         <v>85</v>
       </c>
@@ -4306,12 +4451,12 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-10)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -4351,6 +4496,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J71" t="n">
         <v>38</v>
       </c>
@@ -4361,12 +4511,12 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-30)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -4406,6 +4556,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J72" t="n">
         <v>279</v>
       </c>
@@ -4416,12 +4571,12 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-10-12)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -4461,6 +4616,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J73" t="n">
         <v>273</v>
       </c>
@@ -4471,12 +4631,12 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-30)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -4516,6 +4676,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J74" t="n">
         <v>296</v>
       </c>
@@ -4526,12 +4691,12 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-30)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -4571,6 +4736,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J75" t="n">
         <v>83</v>
       </c>
@@ -4581,12 +4751,12 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-10)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -4626,6 +4796,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J76" t="n">
         <v>300</v>
       </c>
@@ -4636,12 +4811,12 @@
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-30)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -4691,12 +4866,12 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-30)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -4746,12 +4921,12 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-30)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -4801,12 +4976,12 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-30)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -4856,12 +5031,12 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-10)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -4911,12 +5086,12 @@
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-10)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -4966,12 +5141,12 @@
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-30)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -5021,12 +5196,12 @@
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-30)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -5076,12 +5251,12 @@
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-30)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -5131,12 +5306,12 @@
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-30)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -5186,12 +5361,12 @@
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-30)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -5241,12 +5416,12 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-30)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -5296,12 +5471,12 @@
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-30)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -5351,12 +5526,12 @@
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-10)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -5406,12 +5581,12 @@
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-30)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -5851,12 +6026,12 @@
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-30)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -6021,12 +6196,12 @@
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>A_UPLOADER</t>
+          <t>PLUS_RECENT_PRESENT</t>
         </is>
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>1 rapport(s) existant(s)</t>
+          <t>Rapport de gestion Août 2026 (2026-09-30)</t>
         </is>
       </c>
     </row>
@@ -6956,12 +7131,12 @@
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-11)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -7011,12 +7186,12 @@
       </c>
       <c r="L119" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M119" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-11)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -7121,12 +7296,12 @@
       </c>
       <c r="L121" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-11)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -7291,7 +7466,7 @@
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-30); Fiche mensuelle Août 2026 (2026-08-31)</t>
+          <t>Rapport de gestion Août 2026 (2026-09-30)</t>
         </is>
       </c>
     </row>
@@ -7506,12 +7681,12 @@
       </c>
       <c r="L128" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t>Fiche mensuelle Août 2026 (2026-08-31)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -7671,12 +7846,12 @@
       </c>
       <c r="L131" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-30)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -7731,7 +7906,7 @@
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-11); Fiche mensuelle Août 2026 (2026-08-31)</t>
+          <t>Rapport de Gestion Août 2026 (2026-09-11)</t>
         </is>
       </c>
     </row>
@@ -8556,12 +8731,12 @@
       </c>
       <c r="L147" t="inlineStr">
         <is>
-          <t>A_UPLOADER</t>
+          <t>PLUS_RECENT_PRESENT</t>
         </is>
       </c>
       <c r="M147" t="inlineStr">
         <is>
-          <t>2 rapport(s) existant(s)</t>
+          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
         </is>
       </c>
     </row>
@@ -8776,12 +8951,12 @@
       </c>
       <c r="L151" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-29)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -8886,12 +9061,12 @@
       </c>
       <c r="L153" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M153" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-29)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -8941,12 +9116,12 @@
       </c>
       <c r="L154" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M154" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-29)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -8996,12 +9171,12 @@
       </c>
       <c r="L155" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M155" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-29)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -9051,12 +9226,12 @@
       </c>
       <c r="L156" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-29)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -9106,12 +9281,12 @@
       </c>
       <c r="L157" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M157" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-29)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -9161,12 +9336,12 @@
       </c>
       <c r="L158" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M158" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-29)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -9326,12 +9501,12 @@
       </c>
       <c r="L161" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M161" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-29)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -9436,12 +9611,12 @@
       </c>
       <c r="L163" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M163" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-29)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -9491,12 +9666,12 @@
       </c>
       <c r="L164" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M164" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-29)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -9546,12 +9721,12 @@
       </c>
       <c r="L165" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-29)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -9601,12 +9776,12 @@
       </c>
       <c r="L166" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-29)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -9711,12 +9886,12 @@
       </c>
       <c r="L168" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-29)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -9766,12 +9941,12 @@
       </c>
       <c r="L169" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-29)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -9821,12 +9996,12 @@
       </c>
       <c r="L170" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M170" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-29)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -9876,12 +10051,12 @@
       </c>
       <c r="L171" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-29)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -10261,12 +10436,12 @@
       </c>
       <c r="L178" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -10316,12 +10491,12 @@
       </c>
       <c r="L179" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M179" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -10481,12 +10656,12 @@
       </c>
       <c r="L182" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>Rapport de gestion Juin 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -10536,12 +10711,12 @@
       </c>
       <c r="L183" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M183" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -10591,12 +10766,12 @@
       </c>
       <c r="L184" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>Rapport de gestion Juin 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -10646,12 +10821,12 @@
       </c>
       <c r="L185" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-30)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -11636,12 +11811,12 @@
       </c>
       <c r="L203" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M203" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-23)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -11691,12 +11866,12 @@
       </c>
       <c r="L204" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M204" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-23)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -11746,12 +11921,12 @@
       </c>
       <c r="L205" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M205" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-23)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -12521,12 +12696,12 @@
       </c>
       <c r="L219" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M219" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-24)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -12576,12 +12751,12 @@
       </c>
       <c r="L220" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M220" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-24)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -12631,12 +12806,12 @@
       </c>
       <c r="L221" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M221" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-24)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -12686,12 +12861,12 @@
       </c>
       <c r="L222" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M222" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-24)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -12741,12 +12916,12 @@
       </c>
       <c r="L223" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M223" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-24)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -12796,12 +12971,12 @@
       </c>
       <c r="L224" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M224" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-24)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -12851,12 +13026,12 @@
       </c>
       <c r="L225" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M225" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-24)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -12906,12 +13081,12 @@
       </c>
       <c r="L226" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M226" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-24)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -12961,12 +13136,12 @@
       </c>
       <c r="L227" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M227" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-24)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -13016,12 +13191,12 @@
       </c>
       <c r="L228" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M228" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-24)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -13071,12 +13246,12 @@
       </c>
       <c r="L229" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M229" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-24)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -13126,12 +13301,12 @@
       </c>
       <c r="L230" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M230" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-24)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -13181,12 +13356,12 @@
       </c>
       <c r="L231" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M231" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-24)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -13236,12 +13411,12 @@
       </c>
       <c r="L232" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M232" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-24)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -13291,12 +13466,12 @@
       </c>
       <c r="L233" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M233" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-24)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -13346,12 +13521,12 @@
       </c>
       <c r="L234" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M234" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-24)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -13401,12 +13576,12 @@
       </c>
       <c r="L235" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M235" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-24)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -13456,12 +13631,12 @@
       </c>
       <c r="L236" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M236" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-24)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -14116,12 +14291,12 @@
       </c>
       <c r="L248" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M248" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-15)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -14171,12 +14346,12 @@
       </c>
       <c r="L249" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M249" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-15)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -14226,12 +14401,12 @@
       </c>
       <c r="L250" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M250" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-15)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -14281,12 +14456,12 @@
       </c>
       <c r="L251" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M251" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-15)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -14336,12 +14511,12 @@
       </c>
       <c r="L252" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M252" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-25)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -14391,12 +14566,12 @@
       </c>
       <c r="L253" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M253" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-25)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -14726,12 +14901,12 @@
       </c>
       <c r="L259" t="inlineStr">
         <is>
-          <t>A_UPLOADER</t>
+          <t>PLUS_RECENT_PRESENT</t>
         </is>
       </c>
       <c r="M259" t="inlineStr">
         <is>
-          <t>1 rapport(s) existant(s)</t>
+          <t>Rapport de gestion Mars 2026 (2026-09-28)</t>
         </is>
       </c>
     </row>
@@ -14896,12 +15071,12 @@
       </c>
       <c r="L262" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M262" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-25)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -15011,12 +15186,12 @@
       </c>
       <c r="L264" t="inlineStr">
         <is>
-          <t>A_UPLOADER</t>
+          <t>PLUS_RECENT_PRESENT</t>
         </is>
       </c>
       <c r="M264" t="inlineStr">
         <is>
-          <t>1 rapport(s) existant(s)</t>
+          <t>Rapport de gestion Août 2026 (2026-08-31)</t>
         </is>
       </c>
     </row>
@@ -15396,12 +15571,12 @@
       </c>
       <c r="L271" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M271" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Juillet 2026 (2026-09-11)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -15451,12 +15626,12 @@
       </c>
       <c r="L272" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M272" t="inlineStr">
         <is>
-          <t>Rapport mensuel (2026-09-08)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -15506,12 +15681,12 @@
       </c>
       <c r="L273" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M273" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Juillet 2026 (2026-09-11)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -15616,12 +15791,12 @@
       </c>
       <c r="L275" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M275" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Juillet 2026 (2026-09-11)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -15671,12 +15846,12 @@
       </c>
       <c r="L276" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M276" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Juillet 2026 (2026-09-11)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -15726,12 +15901,12 @@
       </c>
       <c r="L277" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M277" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Juillet 2026 (2026-09-11)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -15781,12 +15956,12 @@
       </c>
       <c r="L278" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M278" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Juillet 2026 (2026-09-11)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -15841,12 +16016,12 @@
       </c>
       <c r="L279" t="inlineStr">
         <is>
-          <t>A_UPLOADER</t>
+          <t>PLUS_RECENT_PRESENT</t>
         </is>
       </c>
       <c r="M279" t="inlineStr">
         <is>
-          <t>2 rapport(s) existant(s)</t>
+          <t>Rapport de Gestion Juillet 2026 (2026-09-11)</t>
         </is>
       </c>
     </row>
@@ -15896,12 +16071,12 @@
       </c>
       <c r="L280" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M280" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Juillet 2026 (2026-09-11)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -15951,12 +16126,12 @@
       </c>
       <c r="L281" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M281" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Juillet 2026 (2026-09-11)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -16061,12 +16236,12 @@
       </c>
       <c r="L283" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M283" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -16561,12 +16736,12 @@
       </c>
       <c r="L292" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M292" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -17991,12 +18166,12 @@
       </c>
       <c r="L318" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M318" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -18101,12 +18276,12 @@
       </c>
       <c r="L320" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M320" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -18706,12 +18881,12 @@
       </c>
       <c r="L331" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M331" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-14)</t>
+          <t>3 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -18816,12 +18991,12 @@
       </c>
       <c r="L333" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M333" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-14)</t>
+          <t>3 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -18871,12 +19046,12 @@
       </c>
       <c r="L334" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M334" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-14)</t>
+          <t>3 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -18926,12 +19101,12 @@
       </c>
       <c r="L335" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M335" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-14)</t>
+          <t>3 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -18981,12 +19156,12 @@
       </c>
       <c r="L336" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M336" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-14)</t>
+          <t>3 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -19091,12 +19266,12 @@
       </c>
       <c r="L338" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M338" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-14)</t>
+          <t>3 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -19311,12 +19486,12 @@
       </c>
       <c r="L342" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M342" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-14)</t>
+          <t>3 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -19806,12 +19981,12 @@
       </c>
       <c r="L351" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M351" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -19916,12 +20091,12 @@
       </c>
       <c r="L353" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M353" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -19971,12 +20146,12 @@
       </c>
       <c r="L354" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M354" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -20081,12 +20256,12 @@
       </c>
       <c r="L356" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M356" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -20136,12 +20311,12 @@
       </c>
       <c r="L357" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M357" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -20301,12 +20476,12 @@
       </c>
       <c r="L360" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M360" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -20411,12 +20586,12 @@
       </c>
       <c r="L362" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M362" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -20521,12 +20696,12 @@
       </c>
       <c r="L364" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M364" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -21071,12 +21246,12 @@
       </c>
       <c r="L374" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M374" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -21126,12 +21301,12 @@
       </c>
       <c r="L375" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M375" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -21223,12 +21398,12 @@
       </c>
       <c r="L377" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M377" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -21278,12 +21453,12 @@
       </c>
       <c r="L378" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M378" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -21430,12 +21605,12 @@
       </c>
       <c r="L381" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M381" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -21485,12 +21660,12 @@
       </c>
       <c r="L382" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M382" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -21540,12 +21715,12 @@
       </c>
       <c r="L383" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M383" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -21595,12 +21770,12 @@
       </c>
       <c r="L384" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M384" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -21650,12 +21825,12 @@
       </c>
       <c r="L385" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M385" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -21705,12 +21880,12 @@
       </c>
       <c r="L386" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M386" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -21815,12 +21990,12 @@
       </c>
       <c r="L388" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M388" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -21980,12 +22155,12 @@
       </c>
       <c r="L391" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M391" t="inlineStr">
         <is>
-          <t>DIC (Document d'informations clés) (2026-09-30); Rapport de gestion Août 2026 (2026-09-30)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -22970,12 +23145,12 @@
       </c>
       <c r="L409" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M409" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -23025,12 +23200,12 @@
       </c>
       <c r="L410" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M410" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -23080,12 +23255,12 @@
       </c>
       <c r="L411" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M411" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -23740,12 +23915,12 @@
       </c>
       <c r="L423" t="inlineStr">
         <is>
-          <t>DEJA_PRESENT</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M423" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-30)</t>
+          <t>1 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Upload invest-law.eu terminé : 250 factsheets, note de session
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T5bmrEsYEKdmqU5ckZhZrJ
</commit_message>
<xml_diff>
--- a/INVESTLAW/MANIFEST_UPLOAD.xlsx
+++ b/INVESTLAW/MANIFEST_UPLOAD.xlsx
@@ -4856,6 +4856,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J77" t="n">
         <v>282</v>
       </c>
@@ -4911,6 +4916,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J78" t="n">
         <v>283</v>
       </c>
@@ -4966,6 +4976,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J79" t="n">
         <v>291</v>
       </c>
@@ -5021,6 +5036,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J80" t="n">
         <v>84</v>
       </c>
@@ -5076,6 +5096,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J81" t="n">
         <v>88</v>
       </c>
@@ -5131,6 +5156,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J82" t="n">
         <v>276</v>
       </c>
@@ -5186,6 +5216,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J83" t="n">
         <v>304</v>
       </c>
@@ -5241,6 +5276,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J84" t="n">
         <v>317</v>
       </c>
@@ -5296,6 +5336,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J85" t="n">
         <v>302</v>
       </c>
@@ -5351,6 +5396,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J86" t="n">
         <v>313</v>
       </c>
@@ -5406,6 +5456,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J87" t="n">
         <v>49</v>
       </c>
@@ -5461,6 +5516,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J88" t="n">
         <v>316</v>
       </c>
@@ -5516,6 +5576,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J89" t="n">
         <v>86</v>
       </c>
@@ -5571,6 +5636,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J90" t="n">
         <v>311</v>
       </c>
@@ -5686,6 +5756,11 @@
           <t>Texte PDF brouillé : ISIN vérifié par décodage</t>
         </is>
       </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J92" t="n">
         <v>448</v>
       </c>
@@ -5741,6 +5816,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J93" t="n">
         <v>452</v>
       </c>
@@ -5796,6 +5876,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J94" t="n">
         <v>60</v>
       </c>
@@ -5851,6 +5936,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J95" t="n">
         <v>451</v>
       </c>
@@ -5906,6 +5996,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J96" t="n">
         <v>47</v>
       </c>
@@ -6016,6 +6111,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J98" t="n">
         <v>460</v>
       </c>
@@ -6296,6 +6396,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J103" t="n">
         <v>449</v>
       </c>
@@ -6351,6 +6456,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J104" t="n">
         <v>450</v>
       </c>
@@ -6406,6 +6516,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J105" t="n">
         <v>462</v>
       </c>
@@ -7121,6 +7236,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J118" t="n">
         <v>5</v>
       </c>
@@ -7176,6 +7296,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J119" t="n">
         <v>8</v>
       </c>
@@ -7286,6 +7411,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J121" t="n">
         <v>94</v>
       </c>
@@ -7506,6 +7636,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J125" t="n">
         <v>93</v>
       </c>
@@ -7671,6 +7806,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J128" t="n">
         <v>91</v>
       </c>
@@ -7836,6 +7976,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J131" t="n">
         <v>464</v>
       </c>
@@ -8276,6 +8421,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J139" t="n">
         <v>486</v>
       </c>
@@ -8496,6 +8646,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J143" t="n">
         <v>490</v>
       </c>
@@ -8551,6 +8706,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J144" t="n">
         <v>493</v>
       </c>
@@ -8606,6 +8766,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J145" t="n">
         <v>494</v>
       </c>
@@ -8661,6 +8826,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J146" t="n">
         <v>262</v>
       </c>
@@ -8941,6 +9111,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J151" t="n">
         <v>499</v>
       </c>
@@ -9051,6 +9226,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J153" t="n">
         <v>514</v>
       </c>
@@ -9106,6 +9286,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J154" t="n">
         <v>502</v>
       </c>
@@ -9161,6 +9346,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J155" t="n">
         <v>497</v>
       </c>
@@ -9216,6 +9406,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J156" t="n">
         <v>500</v>
       </c>
@@ -9271,6 +9466,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J157" t="n">
         <v>498</v>
       </c>
@@ -9326,6 +9526,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J158" t="n">
         <v>503</v>
       </c>
@@ -9491,6 +9696,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J161" t="n">
         <v>504</v>
       </c>
@@ -9601,6 +9811,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J163" t="n">
         <v>63</v>
       </c>
@@ -9656,6 +9871,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J164" t="n">
         <v>54</v>
       </c>
@@ -9711,6 +9931,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J165" t="n">
         <v>513</v>
       </c>
@@ -9766,6 +9991,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J166" t="n">
         <v>512</v>
       </c>
@@ -9876,6 +10106,11 @@
           <t>DE</t>
         </is>
       </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J168" t="n">
         <v>16</v>
       </c>
@@ -9931,6 +10166,11 @@
           <t>DE</t>
         </is>
       </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J169" t="n">
         <v>109</v>
       </c>
@@ -9986,6 +10226,11 @@
           <t>DE</t>
         </is>
       </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J170" t="n">
         <v>110</v>
       </c>
@@ -10041,6 +10286,11 @@
           <t>DE</t>
         </is>
       </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J171" t="n">
         <v>111</v>
       </c>
@@ -10096,6 +10346,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J172" t="n">
         <v>516</v>
       </c>
@@ -10426,6 +10681,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J178" t="n">
         <v>428</v>
       </c>
@@ -10481,6 +10741,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J179" t="n">
         <v>429</v>
       </c>
@@ -10536,6 +10801,11 @@
           <t>NL</t>
         </is>
       </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J180" t="n">
         <v>383</v>
       </c>
@@ -10591,6 +10861,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J181" t="n">
         <v>363</v>
       </c>
@@ -10646,6 +10921,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J182" t="n">
         <v>416</v>
       </c>
@@ -10701,6 +10981,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J183" t="n">
         <v>414</v>
       </c>
@@ -10756,6 +11041,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J184" t="n">
         <v>415</v>
       </c>
@@ -10811,6 +11101,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J185" t="n">
         <v>57</v>
       </c>
@@ -10921,6 +11216,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J187" t="n">
         <v>518</v>
       </c>
@@ -10976,6 +11276,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J188" t="n">
         <v>519</v>
       </c>
@@ -11031,6 +11336,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J189" t="n">
         <v>521</v>
       </c>
@@ -11086,6 +11396,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J190" t="n">
         <v>520</v>
       </c>
@@ -11471,6 +11786,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J197" t="n">
         <v>52</v>
       </c>
@@ -11526,6 +11846,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J198" t="n">
         <v>253</v>
       </c>
@@ -11801,6 +12126,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J203" t="n">
         <v>265</v>
       </c>
@@ -11856,6 +12186,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J204" t="n">
         <v>264</v>
       </c>
@@ -11911,6 +12246,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J205" t="n">
         <v>263</v>
       </c>
@@ -11971,6 +12311,11 @@
           <t>Document ancien (&gt;3 mois)</t>
         </is>
       </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J206" t="n">
         <v>267</v>
       </c>
@@ -12246,6 +12591,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J211" t="n">
         <v>274</v>
       </c>
@@ -12356,6 +12706,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J213" t="n">
         <v>343</v>
       </c>
@@ -12411,6 +12766,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J214" t="n">
         <v>345</v>
       </c>
@@ -12466,6 +12826,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J215" t="n">
         <v>266</v>
       </c>
@@ -12521,6 +12886,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J216" t="n">
         <v>280</v>
       </c>
@@ -12576,6 +12946,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J217" t="n">
         <v>67</v>
       </c>
@@ -12631,6 +13006,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J218" t="n">
         <v>281</v>
       </c>
@@ -12686,6 +13066,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J219" t="n">
         <v>289</v>
       </c>
@@ -12741,6 +13126,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J220" t="n">
         <v>14</v>
       </c>
@@ -12796,6 +13186,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J221" t="n">
         <v>293</v>
       </c>
@@ -12851,6 +13246,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J222" t="n">
         <v>285</v>
       </c>
@@ -12906,6 +13306,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J223" t="n">
         <v>69</v>
       </c>
@@ -12961,6 +13366,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J224" t="n">
         <v>299</v>
       </c>
@@ -13016,6 +13426,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J225" t="n">
         <v>284</v>
       </c>
@@ -13071,6 +13486,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J226" t="n">
         <v>288</v>
       </c>
@@ -13126,6 +13546,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J227" t="n">
         <v>290</v>
       </c>
@@ -13181,6 +13606,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J228" t="n">
         <v>48</v>
       </c>
@@ -13236,6 +13666,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J229" t="n">
         <v>294</v>
       </c>
@@ -13291,6 +13726,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J230" t="n">
         <v>297</v>
       </c>
@@ -13346,6 +13786,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J231" t="n">
         <v>298</v>
       </c>
@@ -13401,6 +13846,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J232" t="n">
         <v>51</v>
       </c>
@@ -13456,6 +13906,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J233" t="n">
         <v>292</v>
       </c>
@@ -13511,6 +13966,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J234" t="n">
         <v>286</v>
       </c>
@@ -13566,6 +14026,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J235" t="n">
         <v>287</v>
       </c>
@@ -13621,6 +14086,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J236" t="n">
         <v>295</v>
       </c>
@@ -14116,6 +14586,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J245" t="n">
         <v>463</v>
       </c>
@@ -14281,6 +14756,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J248" t="n">
         <v>115</v>
       </c>
@@ -14336,6 +14816,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J249" t="n">
         <v>112</v>
       </c>
@@ -14391,6 +14876,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J250" t="n">
         <v>114</v>
       </c>
@@ -14446,6 +14936,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J251" t="n">
         <v>113</v>
       </c>
@@ -14501,6 +14996,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J252" t="n">
         <v>314</v>
       </c>
@@ -14556,6 +15056,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J253" t="n">
         <v>315</v>
       </c>
@@ -14611,6 +15116,11 @@
           <t>SV</t>
         </is>
       </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J254" t="n">
         <v>318</v>
       </c>
@@ -14666,6 +15176,11 @@
           <t>SV</t>
         </is>
       </c>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J255" t="n">
         <v>322</v>
       </c>
@@ -14721,6 +15236,11 @@
           <t>SV</t>
         </is>
       </c>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J256" t="n">
         <v>321</v>
       </c>
@@ -14776,6 +15296,11 @@
           <t>SV</t>
         </is>
       </c>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J257" t="n">
         <v>320</v>
       </c>
@@ -15061,6 +15586,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J262" t="n">
         <v>326</v>
       </c>
@@ -15116,6 +15646,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J263" t="n">
         <v>324</v>
       </c>
@@ -15231,6 +15766,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J265" t="n">
         <v>218</v>
       </c>
@@ -15506,6 +16046,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J270" t="n">
         <v>101</v>
       </c>
@@ -15561,6 +16106,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J271" t="n">
         <v>96</v>
       </c>
@@ -15616,6 +16166,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J272" t="n">
         <v>95</v>
       </c>
@@ -15671,6 +16226,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J273" t="n">
         <v>102</v>
       </c>
@@ -15726,6 +16286,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J274" t="n">
         <v>105</v>
       </c>
@@ -15781,6 +16346,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J275" t="n">
         <v>99</v>
       </c>
@@ -15836,6 +16406,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J276" t="n">
         <v>56</v>
       </c>
@@ -15891,6 +16466,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J277" t="n">
         <v>103</v>
       </c>
@@ -15946,6 +16526,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J278" t="n">
         <v>97</v>
       </c>
@@ -16061,6 +16646,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J280" t="n">
         <v>98</v>
       </c>
@@ -16116,6 +16706,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J281" t="n">
         <v>104</v>
       </c>
@@ -16171,6 +16766,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J282" t="n">
         <v>6</v>
       </c>
@@ -16226,6 +16826,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J283" t="n">
         <v>436</v>
       </c>
@@ -16281,6 +16886,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J284" t="n">
         <v>45</v>
       </c>
@@ -16336,6 +16946,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J285" t="n">
         <v>117</v>
       </c>
@@ -16391,6 +17006,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J286" t="n">
         <v>329</v>
       </c>
@@ -16446,6 +17066,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J287" t="n">
         <v>331</v>
       </c>
@@ -16501,6 +17126,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J288" t="n">
         <v>330</v>
       </c>
@@ -16556,6 +17186,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J289" t="n">
         <v>333</v>
       </c>
@@ -16611,6 +17246,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J290" t="n">
         <v>332</v>
       </c>
@@ -16726,6 +17366,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J292" t="n">
         <v>125</v>
       </c>
@@ -16781,6 +17426,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J293" t="n">
         <v>495</v>
       </c>
@@ -16836,6 +17486,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J294" t="n">
         <v>341</v>
       </c>
@@ -16891,6 +17546,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J295" t="n">
         <v>342</v>
       </c>
@@ -16946,6 +17606,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J296" t="n">
         <v>340</v>
       </c>
@@ -17056,6 +17721,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J298" t="n">
         <v>338</v>
       </c>
@@ -17111,6 +17781,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J299" t="n">
         <v>339</v>
       </c>
@@ -17166,6 +17841,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J300" t="n">
         <v>346</v>
       </c>
@@ -17221,6 +17901,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J301" t="n">
         <v>53</v>
       </c>
@@ -17441,6 +18126,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J305" t="n">
         <v>74</v>
       </c>
@@ -17551,6 +18241,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J307" t="n">
         <v>73</v>
       </c>
@@ -17716,6 +18411,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J310" t="n">
         <v>43</v>
       </c>
@@ -18046,6 +18746,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J316" t="n">
         <v>123</v>
       </c>
@@ -18101,6 +18806,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J317" t="n">
         <v>336</v>
       </c>
@@ -18156,6 +18866,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J318" t="n">
         <v>350</v>
       </c>
@@ -18211,6 +18926,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J319" t="n">
         <v>409</v>
       </c>
@@ -18266,6 +18986,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J320" t="n">
         <v>349</v>
       </c>
@@ -18321,6 +19046,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J321" t="n">
         <v>334</v>
       </c>
@@ -18376,6 +19106,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J322" t="n">
         <v>447</v>
       </c>
@@ -18871,6 +19606,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J331" t="n">
         <v>129</v>
       </c>
@@ -18981,6 +19721,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J333" t="n">
         <v>134</v>
       </c>
@@ -19036,6 +19781,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J334" t="n">
         <v>132</v>
       </c>
@@ -19091,6 +19841,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J335" t="n">
         <v>133</v>
       </c>
@@ -19146,6 +19901,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J336" t="n">
         <v>137</v>
       </c>
@@ -19256,6 +20016,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J338" t="n">
         <v>130</v>
       </c>
@@ -19476,6 +20241,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I342" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J342" t="n">
         <v>131</v>
       </c>
@@ -19531,6 +20301,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J343" t="n">
         <v>358</v>
       </c>
@@ -19586,6 +20361,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J344" t="n">
         <v>359</v>
       </c>
@@ -19641,6 +20421,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J345" t="n">
         <v>35</v>
       </c>
@@ -19696,6 +20481,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J346" t="n">
         <v>34</v>
       </c>
@@ -19751,6 +20541,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J347" t="n">
         <v>453</v>
       </c>
@@ -19806,6 +20601,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J348" t="n">
         <v>364</v>
       </c>
@@ -19861,6 +20661,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J349" t="n">
         <v>362</v>
       </c>
@@ -19916,6 +20721,11 @@
           <t>SV</t>
         </is>
       </c>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J350" t="n">
         <v>492</v>
       </c>
@@ -19971,6 +20781,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J351" t="n">
         <v>381</v>
       </c>
@@ -20081,6 +20896,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I353" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J353" t="n">
         <v>368</v>
       </c>
@@ -20136,6 +20956,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I354" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J354" t="n">
         <v>371</v>
       </c>
@@ -20246,6 +21071,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I356" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J356" t="n">
         <v>380</v>
       </c>
@@ -20301,6 +21131,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I357" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J357" t="n">
         <v>366</v>
       </c>
@@ -20466,6 +21301,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J360" t="n">
         <v>370</v>
       </c>
@@ -20576,6 +21416,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I362" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J362" t="n">
         <v>369</v>
       </c>
@@ -20686,6 +21531,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J364" t="n">
         <v>372</v>
       </c>
@@ -20906,6 +21756,11 @@
           <t>DE</t>
         </is>
       </c>
+      <c r="I368" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J368" t="n">
         <v>23</v>
       </c>
@@ -21016,6 +21871,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J370" t="n">
         <v>139</v>
       </c>
@@ -21071,6 +21931,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I371" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J371" t="n">
         <v>365</v>
       </c>
@@ -21236,6 +22101,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I374" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J374" t="n">
         <v>395</v>
       </c>
@@ -21291,6 +22161,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I375" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J375" t="n">
         <v>399</v>
       </c>
@@ -21388,6 +22263,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J377" t="n">
         <v>397</v>
       </c>
@@ -21443,6 +22323,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J378" t="n">
         <v>400</v>
       </c>
@@ -21595,6 +22480,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J381" t="n">
         <v>388</v>
       </c>
@@ -21650,6 +22540,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J382" t="n">
         <v>386</v>
       </c>
@@ -21705,6 +22600,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J383" t="n">
         <v>391</v>
       </c>
@@ -21760,6 +22660,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J384" t="n">
         <v>393</v>
       </c>
@@ -21815,6 +22720,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J385" t="n">
         <v>29</v>
       </c>
@@ -21870,6 +22780,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J386" t="n">
         <v>394</v>
       </c>
@@ -21980,6 +22895,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J388" t="n">
         <v>390</v>
       </c>
@@ -22090,6 +23010,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J390" t="n">
         <v>403</v>
       </c>
@@ -22145,6 +23070,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J391" t="n">
         <v>208</v>
       </c>
@@ -22200,6 +23130,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J392" t="n">
         <v>517</v>
       </c>
@@ -22255,6 +23190,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J393" t="n">
         <v>402</v>
       </c>
@@ -22310,6 +23250,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J394" t="n">
         <v>408</v>
       </c>
@@ -22365,6 +23310,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J395" t="n">
         <v>404</v>
       </c>
@@ -22420,6 +23370,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J396" t="n">
         <v>405</v>
       </c>
@@ -22475,6 +23430,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J397" t="n">
         <v>406</v>
       </c>
@@ -22530,6 +23490,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J398" t="n">
         <v>407</v>
       </c>
@@ -22585,6 +23550,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J399" t="n">
         <v>421</v>
       </c>
@@ -22640,6 +23610,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J400" t="n">
         <v>422</v>
       </c>
@@ -22695,6 +23670,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J401" t="n">
         <v>424</v>
       </c>
@@ -22750,6 +23730,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J402" t="n">
         <v>423</v>
       </c>
@@ -22805,6 +23790,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J403" t="n">
         <v>261</v>
       </c>
@@ -22915,6 +23905,11 @@
           <t>IT</t>
         </is>
       </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J405" t="n">
         <v>433</v>
       </c>
@@ -23025,6 +24020,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J407" t="n">
         <v>461</v>
       </c>
@@ -23080,6 +24080,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J408" t="n">
         <v>434</v>
       </c>
@@ -23135,6 +24140,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J409" t="n">
         <v>439</v>
       </c>
@@ -23190,6 +24200,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J410" t="n">
         <v>438</v>
       </c>
@@ -23245,6 +24260,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J411" t="n">
         <v>437</v>
       </c>
@@ -23300,6 +24320,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J412" t="n">
         <v>441</v>
       </c>
@@ -23355,6 +24380,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J413" t="n">
         <v>442</v>
       </c>
@@ -23520,6 +24550,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J416" t="n">
         <v>106</v>
       </c>
@@ -23575,6 +24610,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J417" t="n">
         <v>15</v>
       </c>
@@ -23630,6 +24670,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J418" t="n">
         <v>107</v>
       </c>
@@ -23685,6 +24730,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J419" t="n">
         <v>198</v>
       </c>
@@ -23740,6 +24790,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J420" t="n">
         <v>197</v>
       </c>
@@ -23795,6 +24850,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J421" t="n">
         <v>196</v>
       </c>
@@ -23850,6 +24910,11 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J422" t="n">
         <v>59</v>
       </c>
@@ -23903,6 +24968,11 @@
       <c r="G423" t="inlineStr">
         <is>
           <t>FR</t>
+        </is>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
         </is>
       </c>
       <c r="J423" t="n">

</xml_diff>

<commit_message>
Harmonisation appliquée (82 rapports), upload ACATIS, détection des doublons élargie aux « Fiche mensuelle »
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T5bmrEsYEKdmqU5ckZhZrJ
</commit_message>
<xml_diff>
--- a/INVESTLAW/MANIFEST_UPLOAD.xlsx
+++ b/INVESTLAW/MANIFEST_UPLOAD.xlsx
@@ -596,6 +596,11 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J3" t="n">
         <v>207</v>
       </c>
@@ -606,12 +611,12 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>A_VERIFIER</t>
+          <t>A_UPLOADER</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>rapport de gestion (2026-09-28)</t>
+          <t>2 rapport(s) existant(s)</t>
         </is>
       </c>
     </row>
@@ -8901,12 +8906,12 @@
       </c>
       <c r="L147" t="inlineStr">
         <is>
-          <t>PLUS_RECENT_PRESENT</t>
+          <t>DEJA_PRESENT</t>
         </is>
       </c>
       <c r="M147" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
+          <t>Rapport de gestion Février 2026 (2026-02-27)</t>
         </is>
       </c>
     </row>
@@ -16606,7 +16611,7 @@
       </c>
       <c r="M279" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Juillet 2026 (2026-09-11)</t>
+          <t>Rapport de Gestion Juillet 2026 (2026-09-11); Rapport de gestion Mai 2026 (2026-05-31)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recherche des factsheets manquantes : 9 trouvées et rangées, page d'audit mise à jour
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T5bmrEsYEKdmqU5ckZhZrJ
</commit_message>
<xml_diff>
--- a/INVESTLAW/MANIFEST_UPLOAD.xlsx
+++ b/INVESTLAW/MANIFEST_UPLOAD.xlsx
@@ -419,8 +419,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M423"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:M432"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
@@ -24999,6 +24999,366 @@
         </is>
       </c>
     </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>LU2059537956</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>FFG GLOBAL EQUITY CONVICTIONS I EUR</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>Funds For Good (FFG)</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>Rapport de Gestion Août 2026</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>FUNDS_FOR_GOOD_FFG/LU2059537956/LU2059537956__Factsheet_FR_2026-08-31.pdf</t>
+        </is>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="J424" t="n">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>LU2736456752</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>FFG GLOBAL EQUITIES LOW CARBON I EUR</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>Funds For Good (FFG)</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>Rapport de Gestion Août 2026</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t>FUNDS_FOR_GOOD_FFG/LU2736456752/LU2736456752__Factsheet_FR_2026-08-31.pdf</t>
+        </is>
+      </c>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="J425" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>LU2612532833</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>FFG BLI GLOBAL IMPACT EQUITIES I EUR</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>Funds For Good (FFG)</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>Rapport de Gestion Août 2026</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t>FUNDS_FOR_GOOD_FFG/LU2612532833/LU2612532833__Factsheet_FR_2026-08-31.pdf</t>
+        </is>
+      </c>
+      <c r="G426" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="J426" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>LU2612531868</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>FFG BLI AMERICAN IMPACT EQUITIES I USD</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>Funds For Good (FFG)</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>Rapport de Gestion Août 2026</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>FUNDS_FOR_GOOD_FFG/LU2612531868/LU2612531868__Factsheet_FR_2026-08-31.pdf</t>
+        </is>
+      </c>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="J427" t="n">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>LU2612531355</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>FFG BLI EUROPEAN IMPACT EQUITIES I EUR</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>Funds For Good (FFG)</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>Rapport de Gestion Août 2026</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>FUNDS_FOR_GOOD_FFG/LU2612531355/LU2612531355__Factsheet_FR_2026-08-31.pdf</t>
+        </is>
+      </c>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="J428" t="n">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>LU1697917166</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>FFG GLOBAL FLEXIBLE CONVICTIONS I EUR</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>Funds For Good (FFG)</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>Rapport de Gestion Août 2026</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>FUNDS_FOR_GOOD_FFG/LU1697917166/LU1697917166__Factsheet_FR_2026-08-31.pdf</t>
+        </is>
+      </c>
+      <c r="G429" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="J429" t="n">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>LU0945617289</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>FFG GLOBAL DEFENSIVE I EUR</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>Funds For Good (FFG)</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>Rapport de Gestion Août 2026</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t>FUNDS_FOR_GOOD_FFG/LU0945617289/LU0945617289__Factsheet_FR_2026-08-31.pdf</t>
+        </is>
+      </c>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="J430" t="n">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>LU1502282632</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>CANDRIAM EQS L ROBOTIC &amp; INNOVATIVE TECHNO C EUR</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>Candriam</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>Rapport de Gestion Septembre 2026</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>CANDRIAM/LU1502282632/LU1502282632__Factsheet_EN_2026-09-30.pdf</t>
+        </is>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="J431" t="n">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>FR001400SJA2</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>IVO IG 2030 R EUR</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>Ivo Capital Partners</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>Rapport de Gestion Août 2026</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>IVO_CAPITAL_PARTNERS/FR001400SJA2/FR001400SJA2__Factsheet_FR_2026-08-31.pdf</t>
+        </is>
+      </c>
+      <c r="G432" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="J432" t="n">
+        <v>278</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I423"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Upload des 9 factsheets trouvées ; Alken et Waterloo écartés
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T5bmrEsYEKdmqU5ckZhZrJ
</commit_message>
<xml_diff>
--- a/INVESTLAW/MANIFEST_UPLOAD.xlsx
+++ b/INVESTLAW/MANIFEST_UPLOAD.xlsx
@@ -420,7 +420,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M432"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
@@ -7601,7 +7601,7 @@
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>Rapport de gestion Août 2026 (2026-09-30)</t>
+          <t>Rapport de gestion Août 2026 (2026-09-30); Fiche mensuelle Août 2026 (2026-08-31)</t>
         </is>
       </c>
     </row>
@@ -8056,7 +8056,7 @@
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>Rapport de Gestion Août 2026 (2026-09-11)</t>
+          <t>Rapport de Gestion Août 2026 (2026-09-11); Fiche mensuelle Août 2026 (2026-08-31)</t>
         </is>
       </c>
     </row>
@@ -22388,9 +22388,22 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="J379" t="n">
+        <v>387</v>
+      </c>
+      <c r="K379" t="inlineStr">
+        <is>
+          <t>R-CO GOLD MINING EUR C</t>
+        </is>
+      </c>
       <c r="L379" t="inlineStr">
         <is>
-          <t>FONDS_ABSENT</t>
+          <t>DEJA_PRESENT</t>
+        </is>
+      </c>
+      <c r="M379" t="inlineStr">
+        <is>
+          <t>Rapport de gestion Août 2026 (2026-09-28)</t>
         </is>
       </c>
     </row>
@@ -25035,9 +25048,29 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I424" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J424" t="n">
         <v>199</v>
       </c>
+      <c r="K424" t="inlineStr">
+        <is>
+          <t>FFG GLOBAL EQUITY CONVICTIONS I EUR</t>
+        </is>
+      </c>
+      <c r="L424" t="inlineStr">
+        <is>
+          <t>A_UPLOADER</t>
+        </is>
+      </c>
+      <c r="M424" t="inlineStr">
+        <is>
+          <t>1 rapport(s) existant(s)</t>
+        </is>
+      </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
@@ -25075,9 +25108,29 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J425" t="n">
         <v>200</v>
       </c>
+      <c r="K425" t="inlineStr">
+        <is>
+          <t>FFG GLOBAL EQUITIES LOW CARBON I EUR</t>
+        </is>
+      </c>
+      <c r="L425" t="inlineStr">
+        <is>
+          <t>A_UPLOADER</t>
+        </is>
+      </c>
+      <c r="M425" t="inlineStr">
+        <is>
+          <t>1 rapport(s) existant(s)</t>
+        </is>
+      </c>
     </row>
     <row r="426">
       <c r="A426" t="inlineStr">
@@ -25115,9 +25168,29 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J426" t="n">
         <v>201</v>
       </c>
+      <c r="K426" t="inlineStr">
+        <is>
+          <t>FFG BLI GLOBAL IMPACT EQUITIES I EUR</t>
+        </is>
+      </c>
+      <c r="L426" t="inlineStr">
+        <is>
+          <t>A_UPLOADER</t>
+        </is>
+      </c>
+      <c r="M426" t="inlineStr">
+        <is>
+          <t>1 rapport(s) existant(s)</t>
+        </is>
+      </c>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
@@ -25155,9 +25228,29 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I427" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J427" t="n">
         <v>202</v>
       </c>
+      <c r="K427" t="inlineStr">
+        <is>
+          <t>FFG BLI AMERICAN IMPACT EQUITIES I USD</t>
+        </is>
+      </c>
+      <c r="L427" t="inlineStr">
+        <is>
+          <t>A_UPLOADER</t>
+        </is>
+      </c>
+      <c r="M427" t="inlineStr">
+        <is>
+          <t>1 rapport(s) existant(s)</t>
+        </is>
+      </c>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
@@ -25195,9 +25288,29 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I428" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J428" t="n">
         <v>203</v>
       </c>
+      <c r="K428" t="inlineStr">
+        <is>
+          <t>FFG BLI EUROPEAN IMPACT EQUITIES I EUR</t>
+        </is>
+      </c>
+      <c r="L428" t="inlineStr">
+        <is>
+          <t>A_UPLOADER</t>
+        </is>
+      </c>
+      <c r="M428" t="inlineStr">
+        <is>
+          <t>1 rapport(s) existant(s)</t>
+        </is>
+      </c>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
@@ -25235,9 +25348,29 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I429" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J429" t="n">
         <v>204</v>
       </c>
+      <c r="K429" t="inlineStr">
+        <is>
+          <t>FFG GLOBAL FLEXIBLE CONVICTIONS I EUR</t>
+        </is>
+      </c>
+      <c r="L429" t="inlineStr">
+        <is>
+          <t>A_UPLOADER</t>
+        </is>
+      </c>
+      <c r="M429" t="inlineStr">
+        <is>
+          <t>1 rapport(s) existant(s)</t>
+        </is>
+      </c>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
@@ -25275,9 +25408,29 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I430" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J430" t="n">
         <v>205</v>
       </c>
+      <c r="K430" t="inlineStr">
+        <is>
+          <t>FFG GLOBAL DEFENSIVE I EUR</t>
+        </is>
+      </c>
+      <c r="L430" t="inlineStr">
+        <is>
+          <t>A_UPLOADER</t>
+        </is>
+      </c>
+      <c r="M430" t="inlineStr">
+        <is>
+          <t>0 rapport(s) existant(s)</t>
+        </is>
+      </c>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
@@ -25315,9 +25468,29 @@
           <t>EN</t>
         </is>
       </c>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J431" t="n">
         <v>250</v>
       </c>
+      <c r="K431" t="inlineStr">
+        <is>
+          <t>CANDRIAM EQS L ROBOTIC &amp; INNOVATIVE TECHNO C EUR</t>
+        </is>
+      </c>
+      <c r="L431" t="inlineStr">
+        <is>
+          <t>A_UPLOADER</t>
+        </is>
+      </c>
+      <c r="M431" t="inlineStr">
+        <is>
+          <t>1 rapport(s) existant(s)</t>
+        </is>
+      </c>
     </row>
     <row r="432">
       <c r="A432" t="inlineStr">
@@ -25355,8 +25528,28 @@
           <t>FR</t>
         </is>
       </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t>UPLOADE</t>
+        </is>
+      </c>
       <c r="J432" t="n">
         <v>278</v>
+      </c>
+      <c r="K432" t="inlineStr">
+        <is>
+          <t>IVO IG 2030 R EUR</t>
+        </is>
+      </c>
+      <c r="L432" t="inlineStr">
+        <is>
+          <t>A_UPLOADER</t>
+        </is>
+      </c>
+      <c r="M432" t="inlineStr">
+        <is>
+          <t>0 rapport(s) existant(s)</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>